<commit_message>
feat(cadrage): Product Vision Board POST PERTURBATION J1 d’EduTutor IA
</commit_message>
<xml_diff>
--- a/docs/cadrage/Product_Vision_Board_EduTutor_IA.xlsx
+++ b/docs/cadrage/Product_Vision_Board_EduTutor_IA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\msi\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F360C1B6-AF5E-468D-B13C-E6C95588EA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{996B4D36-2CB5-4F26-9DB8-CF10503B9566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,13 +46,6 @@
     <t>BUSINESS GOALS</t>
   </si>
   <si>
-    <t xml:space="preserve">• Importer facilement un cours au format PDF de 5 Mo maximum ou saisir directement un texte d’au moins 200 caractères.
-• Générer automatiquement un quiz de 10 QCM en moins de 60 secondes, à partir des notions réellement présentes dans le cours fourni.
-• Proposer une correction automatique avec un score sur 10, l’affichage des bonnes et mauvaises réponses et un retour clair pour l’étudiant.
-• Enregistrer l’historique des quiz, des dates et des scores afin de permettre à l’utilisateur de suivre sa progression dans le temps.
-• Utiliser une intelligence artificielle locale via Ollama pour mieux protéger les cours, limiter les transferts de données vers des services externes et garantir davantage de confidentialité.                        </t>
-  </si>
-  <si>
     <t>• Atteindre environ 1 000 étudiants actifs par semaine dans les six mois suivant le lancement.
 • Obtenir au moins 40 % de rétention à sept jours, afin qu’une part importante des nouveaux utilisateurs revienne utiliser la plateforme.
 • Atteindre un taux de complétion d’au moins 70 % des quiz commencés.
@@ -75,12 +68,6 @@
     <t>5.2. OBJECTIFS DE SATISFACTION ET DE QUALITÉ</t>
   </si>
   <si>
-    <t>• Satisfaction : atteindre un NPS supérieur à 30 d’ici T+9 mois. Ce score permettra d’évaluer la probabilité que les utilisateurs recommandent EduTutor IA à d’autres étudiants ou enseignants.
-• Qualité du contenu : maintenir à moins de 5 % la proportion de quiz signalés pour erreur factuelle, réponse incorrecte, ambiguïté ou question hors sujet. Chaque signalement devra pouvoir être analysé afin d’améliorer les prompts et les contrôles de génération.
-• Expérience utilisateur : obtenir une note moyenne d’au moins 4/5 pour la simplicité de l’interface, la pertinence des questions et l’utilité de la correction.
-• Performance perçue : générer au moins 90 % des quiz en moins de 60 secondes lorsque le document respecte les formats et limites demandés.</t>
-  </si>
-  <si>
     <t>5.3. OBJECTIFS BUSINESS À LONG TERME</t>
   </si>
   <si>
@@ -162,19 +149,67 @@
     <t>EduTutor IA peut fonctionner avec Ollama sur une infrastructure locale ou maîtrisée. Les cours et documents pédagogiques ne sont ainsi pas systématiquement transmis à une API externe. Cette maîtrise des données protège les utilisateurs, limite la dépendance à un fournisseur unique et constitue un argument fort pour les établissements soumis à des obligations de confidentialité et de conformité.</t>
   </si>
   <si>
-    <t xml:space="preserve">Artefact 1/7 </t>
-  </si>
-  <si>
     <t>De nombreux outils d’intelligence artificielle éducative sont surtout conçus pour l’étudiant : il pose une question, obtient un résumé ou génère des fiches. EduTutor IA répond également au besoin des enseignants de produire rapidement des QCM, de contrôler les questions et d’adapter les évaluations à leur contexte pédagogique. Cette complémentarité augmente la valeur de la solution pour un établissemen</t>
   </si>
   <si>
+    <t>Membres : Amani LAYOUNI, Awadi BEDJA MROINKODO SAID, Clément BASTIEN, Rania ZERAMDINI, Taise de Thèse NGANGA YABIE,Badreddine CHEBBOUR</t>
+  </si>
+  <si>
+    <t>Artefact 1/7 — Version v2.0 post‑perturbation J1 · Enseignant cible primaire</t>
+  </si>
+  <si>
+    <t>Version : v2.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Importer facilement un cours au format PDF de 5 Mo maximum ou saisir directement un texte d’au moins 200 caractères.
+• Générer automatiquement un quiz de 10 QCM en moins de 60 secondes, à partir des notions réellement présentes dans le cours fourni.
+• Proposer une correction automatique avec un score sur 10, l’affichage des bonnes et mauvaises réponses et un retour clair pour l’étudiant.
+• Enregistrer l’historique des quiz, des dates et des scores afin de permettre à l’utilisateur de suivre sa progression dans le temps.
+• Ajouter un espace enseignant permettant de consulter la liste des étudiants, leurs derniers scores et leur dernière activité.
+• Signaler clairement les étudiants en difficulté ou inactifs et permettre un filtrage simple.
+• Permettre à l’enseignant d’envoyer un conseil personnalisé à un étudiant.
+• Utiliser une intelligence artificielle locale via Ollama pour mieux protéger les cours, limiter les transferts de données vers des services externes et garantir davantage de confidentialité.                        </t>
+  </si>
+  <si>
+    <t>• Satisfaction : atteindre un NPS supérieur à 30 d’ici T+9 mois. Ce score permettra d’évaluer la probabilité que les utilisateurs recommandent EduTutor IA à d’autres étudiants ou enseignants.
+• Qualité du contenu : maintenir à moins de 5 % la proportion de quiz signalés pour erreur factuelle, réponse incorrecte, ambiguïté ou question hors sujet. Chaque signalement devra pouvoir être analysé afin d’améliorer les prompts et les contrôles de génération.
+• Expérience utilisateur : obtenir une note moyenne d’au moins 4/5 pour la simplicité de l’interface, la pertinence des questions et l’utilité de la correction.
+• Expérience enseignant : permettre à au moins 80 % des enseignants testeurs d’identifier un étudiant en difficulté en moins de trois clics et d’envoyer un conseil sans aide extérieure.
+• Performance perçue : générer au moins 90 % des quiz en moins de 60 secondes lorsque le document respecte les formats et limites demandés.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Étudiant] : Transformer rapidement un cours PDF ou texte en quiz personnalisé, sans perdre du temps à créer les questions manuellement.
+[Étudiant] : Réviser uniquement les notions réellement présentes dans son cours afin d’éviter les questions hors sujet.
+[Étudiant] : Identifier ses lacunes grâce au score, au détail des erreurs et à l’historique de ses quiz.
+[Étudiant] : Comprendre ses mauvaises réponses grâce à une correction claire et progresser avant les examens.
+[Enseignant — cible primaire] : Générer rapidement des QCM adaptés à partir de ses supports de cours.
+[Enseignant — cible primaire] : Consulter les scores, la participation et la dernière activité de ses 28 étudiants.
+[Enseignant — cible primaire] : Repérer rapidement les étudiants en difficulté ou inactifs afin d’intervenir avant le décrochage.
+[Enseignant — cible primaire] : Envoyer un conseil personnalisé à un étudiant selon ses résultats.
+[Établissement - cible tertiare] : Utiliser une solution pédagogique sécurisée, conforme au RGPD et respectueuse de la confidentialité des données.
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>• Cible primaire 1 :</t>
+    </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF222222"/>
-        <rFont val="Carlito"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve">• Cible primaire : </t>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
@@ -196,7 +231,7 @@
         <scheme val="major"/>
       </rPr>
       <t xml:space="preserve"> du supérieur de 18 à 25 ans, de L1 à M2, préparant leurs examens sur ordinateur ou smartphone.
-• Cible secondaire : </t>
+</t>
     </r>
     <r>
       <rPr>
@@ -207,7 +242,8 @@
         <family val="2"/>
         <scheme val="major"/>
       </rPr>
-      <t>enseignants</t>
+      <t xml:space="preserve">
+• Cible primaire 2 : Enseignant·e</t>
     </r>
     <r>
       <rPr>
@@ -217,8 +253,8 @@
         <family val="2"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve"> de lycée, BTS, université ou école supérieure souhaitant créer rapidement des supports d’évaluation.
-• Cible tertiaire : </t>
+      <t xml:space="preserve"> : enseignant de lycée, BTS, université ou école supérieure. Mme Sophie Lefèvre, 42 ans, enseignante en BTS Communication à Lyon, suit 28 étudiants et souhaite consulter leurs scores, repérer ceux qui décrochent et leur envoyer des conseils.
+•</t>
     </r>
     <r>
       <rPr>
@@ -229,7 +265,7 @@
         <family val="2"/>
         <scheme val="major"/>
       </rPr>
-      <t>établissements scolaires</t>
+      <t xml:space="preserve"> Cible tertiaire :</t>
     </r>
     <r>
       <rPr>
@@ -239,33 +275,37 @@
         <family val="2"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve">, écoles supérieures et organismes de formation recherchant un outil conforme au RGPD.
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>établissements scolaires :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </rPr>
+      <t xml:space="preserve"> écoles supérieures et organismes de formation recherchant  une solution pédagogique sécurisée et un outil conforme au RGPD.
 </t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">[Étudiant] : Transformer rapidement un cours PDF ou texte en quiz personnalisé, sans perdre du temps à créer les questions manuellement.
-[Étudiant] : Réviser uniquement les notions réellement présentes dans son cours afin d’éviter les questions hors sujet.
-[Étudiant] : Identifier ses lacunes grâce au score, au détail des erreurs et à l’historique de ses quiz.
-[Étudiant] : Comprendre ses mauvaises réponses grâce à une correction claire et progresser avant les examens.
-[Enseignant] : Générer rapidement des QCM et des supports d’évaluation adaptés au niveau des étudiants.
-[Enseignant] : Réduire le temps consacré à la préparation des évaluations tout en gardant la possibilité de vérifier et modifier les questions.
-[Établissement] : Utiliser une solution pédagogique sécurisée, conforme au RGPD et respectueuse de la confidentialité des données.
-[Établissement] : Conserver la maîtrise des contenus pédagogiques et limiter la dépendance aux services d’intelligence artificielle externes.
-</t>
-  </si>
-  <si>
-    <t>Membres : Amani LAYOUNI, Awadi BEDJA MROINKODO SAID, Clément BASTIEN, Rania ZERAMDINI, Taise de Thèse NGANGA YABIE,Badreddine CHEBBOUR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version : v1.0 (initiale) </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -428,6 +468,13 @@
     <font>
       <sz val="10"/>
       <color rgb="FF222222"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF24303F"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="major"/>
@@ -761,7 +808,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -872,33 +919,36 @@
     <xf numFmtId="0" fontId="7" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -932,7 +982,7 @@
     <xf numFmtId="0" fontId="5" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -957,6 +1007,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="14" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1343,56 +1396,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27.15" customHeight="1">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
     </row>
     <row r="2" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="51"/>
-      <c r="L2" s="51"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
     </row>
     <row r="3" spans="1:12" ht="32.4" customHeight="1">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="54" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
-      <c r="G3" s="53"/>
-      <c r="H3" s="53"/>
-      <c r="I3" s="53"/>
-      <c r="J3" s="53" t="s">
-        <v>46</v>
-      </c>
-      <c r="K3" s="53"/>
-      <c r="L3" s="53"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54" t="s">
+        <v>42</v>
+      </c>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
     </row>
     <row r="5" spans="1:12" ht="19.95" customHeight="1">
       <c r="A5" s="2" t="s">
@@ -1506,22 +1559,22 @@
     </row>
     <row r="13" spans="1:12" ht="17.55" customHeight="1">
       <c r="A13" s="38" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B13" s="39"/>
       <c r="C13" s="40"/>
-      <c r="D13" s="38" t="s">
-        <v>44</v>
+      <c r="D13" s="47" t="s">
+        <v>45</v>
       </c>
       <c r="E13" s="39"/>
       <c r="F13" s="40"/>
       <c r="G13" s="47" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="H13" s="39"/>
       <c r="I13" s="40"/>
-      <c r="J13" s="47" t="s">
-        <v>9</v>
+      <c r="J13" s="48" t="s">
+        <v>8</v>
       </c>
       <c r="K13" s="39"/>
       <c r="L13" s="40"/>
@@ -1778,7 +1831,7 @@
       <c r="K31" s="42"/>
       <c r="L31" s="43"/>
     </row>
-    <row r="32" spans="1:12" ht="30.6" customHeight="1">
+    <row r="32" spans="1:12" ht="107.4" customHeight="1">
       <c r="A32" s="44"/>
       <c r="B32" s="45"/>
       <c r="C32" s="46"/>
@@ -1794,7 +1847,7 @@
     </row>
     <row r="34" spans="1:12" ht="24" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -1809,1130 +1862,1130 @@
       <c r="L34" s="4"/>
     </row>
     <row r="36" spans="1:12" ht="16.8">
-      <c r="A36" s="55" t="s">
+      <c r="A36" s="56" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="57"/>
+      <c r="C36" s="57"/>
+      <c r="D36" s="57"/>
+      <c r="E36" s="57"/>
+      <c r="F36" s="57"/>
+      <c r="G36" s="57"/>
+      <c r="H36" s="57"/>
+      <c r="I36" s="57"/>
+      <c r="J36" s="57"/>
+      <c r="K36" s="57"/>
+      <c r="L36" s="58"/>
+    </row>
+    <row r="37" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A37" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="B36" s="56"/>
-      <c r="C36" s="56"/>
-      <c r="D36" s="56"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="56"/>
-      <c r="G36" s="56"/>
-      <c r="H36" s="56"/>
-      <c r="I36" s="56"/>
-      <c r="J36" s="56"/>
-      <c r="K36" s="56"/>
-      <c r="L36" s="57"/>
-    </row>
-    <row r="37" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A37" s="58" t="s">
+      <c r="B37" s="60"/>
+      <c r="C37" s="60"/>
+      <c r="D37" s="60"/>
+      <c r="E37" s="60"/>
+      <c r="F37" s="60"/>
+      <c r="G37" s="60"/>
+      <c r="H37" s="60"/>
+      <c r="I37" s="60"/>
+      <c r="J37" s="60"/>
+      <c r="K37" s="60"/>
+      <c r="L37" s="61"/>
+    </row>
+    <row r="38" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A38" s="62"/>
+      <c r="B38" s="63"/>
+      <c r="C38" s="63"/>
+      <c r="D38" s="63"/>
+      <c r="E38" s="63"/>
+      <c r="F38" s="63"/>
+      <c r="G38" s="63"/>
+      <c r="H38" s="63"/>
+      <c r="I38" s="63"/>
+      <c r="J38" s="63"/>
+      <c r="K38" s="63"/>
+      <c r="L38" s="64"/>
+    </row>
+    <row r="39" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A39" s="62"/>
+      <c r="B39" s="63"/>
+      <c r="C39" s="63"/>
+      <c r="D39" s="63"/>
+      <c r="E39" s="63"/>
+      <c r="F39" s="63"/>
+      <c r="G39" s="63"/>
+      <c r="H39" s="63"/>
+      <c r="I39" s="63"/>
+      <c r="J39" s="63"/>
+      <c r="K39" s="63"/>
+      <c r="L39" s="64"/>
+    </row>
+    <row r="40" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A40" s="62"/>
+      <c r="B40" s="63"/>
+      <c r="C40" s="63"/>
+      <c r="D40" s="63"/>
+      <c r="E40" s="63"/>
+      <c r="F40" s="63"/>
+      <c r="G40" s="63"/>
+      <c r="H40" s="63"/>
+      <c r="I40" s="63"/>
+      <c r="J40" s="63"/>
+      <c r="K40" s="63"/>
+      <c r="L40" s="64"/>
+    </row>
+    <row r="41" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A41" s="62"/>
+      <c r="B41" s="63"/>
+      <c r="C41" s="63"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="63"/>
+      <c r="F41" s="63"/>
+      <c r="G41" s="63"/>
+      <c r="H41" s="63"/>
+      <c r="I41" s="63"/>
+      <c r="J41" s="63"/>
+      <c r="K41" s="63"/>
+      <c r="L41" s="64"/>
+    </row>
+    <row r="42" spans="1:12" ht="7.8" customHeight="1">
+      <c r="A42" s="62"/>
+      <c r="B42" s="63"/>
+      <c r="C42" s="63"/>
+      <c r="D42" s="63"/>
+      <c r="E42" s="63"/>
+      <c r="F42" s="63"/>
+      <c r="G42" s="63"/>
+      <c r="H42" s="63"/>
+      <c r="I42" s="63"/>
+      <c r="J42" s="63"/>
+      <c r="K42" s="63"/>
+      <c r="L42" s="64"/>
+    </row>
+    <row r="43" spans="1:12" ht="19.2" hidden="1" customHeight="1">
+      <c r="A43" s="65"/>
+      <c r="B43" s="66"/>
+      <c r="C43" s="66"/>
+      <c r="D43" s="66"/>
+      <c r="E43" s="66"/>
+      <c r="F43" s="66"/>
+      <c r="G43" s="66"/>
+      <c r="H43" s="66"/>
+      <c r="I43" s="66"/>
+      <c r="J43" s="66"/>
+      <c r="K43" s="66"/>
+      <c r="L43" s="67"/>
+    </row>
+    <row r="45" spans="1:12" ht="16.8">
+      <c r="A45" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="B37" s="59"/>
-      <c r="C37" s="59"/>
-      <c r="D37" s="59"/>
-      <c r="E37" s="59"/>
-      <c r="F37" s="59"/>
-      <c r="G37" s="59"/>
-      <c r="H37" s="59"/>
-      <c r="I37" s="59"/>
-      <c r="J37" s="59"/>
-      <c r="K37" s="59"/>
-      <c r="L37" s="60"/>
-    </row>
-    <row r="38" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A38" s="61"/>
-      <c r="B38" s="62"/>
-      <c r="C38" s="62"/>
-      <c r="D38" s="62"/>
-      <c r="E38" s="62"/>
-      <c r="F38" s="62"/>
-      <c r="G38" s="62"/>
-      <c r="H38" s="62"/>
-      <c r="I38" s="62"/>
-      <c r="J38" s="62"/>
-      <c r="K38" s="62"/>
-      <c r="L38" s="63"/>
-    </row>
-    <row r="39" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A39" s="61"/>
-      <c r="B39" s="62"/>
-      <c r="C39" s="62"/>
-      <c r="D39" s="62"/>
-      <c r="E39" s="62"/>
-      <c r="F39" s="62"/>
-      <c r="G39" s="62"/>
-      <c r="H39" s="62"/>
-      <c r="I39" s="62"/>
-      <c r="J39" s="62"/>
-      <c r="K39" s="62"/>
-      <c r="L39" s="63"/>
-    </row>
-    <row r="40" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A40" s="61"/>
-      <c r="B40" s="62"/>
-      <c r="C40" s="62"/>
-      <c r="D40" s="62"/>
-      <c r="E40" s="62"/>
-      <c r="F40" s="62"/>
-      <c r="G40" s="62"/>
-      <c r="H40" s="62"/>
-      <c r="I40" s="62"/>
-      <c r="J40" s="62"/>
-      <c r="K40" s="62"/>
-      <c r="L40" s="63"/>
-    </row>
-    <row r="41" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A41" s="61"/>
-      <c r="B41" s="62"/>
-      <c r="C41" s="62"/>
-      <c r="D41" s="62"/>
-      <c r="E41" s="62"/>
-      <c r="F41" s="62"/>
-      <c r="G41" s="62"/>
-      <c r="H41" s="62"/>
-      <c r="I41" s="62"/>
-      <c r="J41" s="62"/>
-      <c r="K41" s="62"/>
-      <c r="L41" s="63"/>
-    </row>
-    <row r="42" spans="1:12" ht="7.8" customHeight="1">
-      <c r="A42" s="61"/>
-      <c r="B42" s="62"/>
-      <c r="C42" s="62"/>
-      <c r="D42" s="62"/>
-      <c r="E42" s="62"/>
-      <c r="F42" s="62"/>
-      <c r="G42" s="62"/>
-      <c r="H42" s="62"/>
-      <c r="I42" s="62"/>
-      <c r="J42" s="62"/>
-      <c r="K42" s="62"/>
-      <c r="L42" s="63"/>
-    </row>
-    <row r="43" spans="1:12" ht="19.2" hidden="1" customHeight="1">
-      <c r="A43" s="64"/>
-      <c r="B43" s="65"/>
-      <c r="C43" s="65"/>
-      <c r="D43" s="65"/>
-      <c r="E43" s="65"/>
-      <c r="F43" s="65"/>
-      <c r="G43" s="65"/>
-      <c r="H43" s="65"/>
-      <c r="I43" s="65"/>
-      <c r="J43" s="65"/>
-      <c r="K43" s="65"/>
-      <c r="L43" s="66"/>
-    </row>
-    <row r="45" spans="1:12" ht="16.8">
-      <c r="A45" s="55" t="s">
+      <c r="B45" s="57"/>
+      <c r="C45" s="57"/>
+      <c r="D45" s="57"/>
+      <c r="E45" s="57"/>
+      <c r="F45" s="57"/>
+      <c r="G45" s="57"/>
+      <c r="H45" s="57"/>
+      <c r="I45" s="57"/>
+      <c r="J45" s="57"/>
+      <c r="K45" s="57"/>
+      <c r="L45" s="58"/>
+    </row>
+    <row r="46" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A46" s="59" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" s="60"/>
+      <c r="C46" s="60"/>
+      <c r="D46" s="60"/>
+      <c r="E46" s="60"/>
+      <c r="F46" s="60"/>
+      <c r="G46" s="60"/>
+      <c r="H46" s="60"/>
+      <c r="I46" s="60"/>
+      <c r="J46" s="60"/>
+      <c r="K46" s="60"/>
+      <c r="L46" s="61"/>
+    </row>
+    <row r="47" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A47" s="62"/>
+      <c r="B47" s="63"/>
+      <c r="C47" s="63"/>
+      <c r="D47" s="63"/>
+      <c r="E47" s="63"/>
+      <c r="F47" s="63"/>
+      <c r="G47" s="63"/>
+      <c r="H47" s="63"/>
+      <c r="I47" s="63"/>
+      <c r="J47" s="63"/>
+      <c r="K47" s="63"/>
+      <c r="L47" s="64"/>
+    </row>
+    <row r="48" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A48" s="62"/>
+      <c r="B48" s="63"/>
+      <c r="C48" s="63"/>
+      <c r="D48" s="63"/>
+      <c r="E48" s="63"/>
+      <c r="F48" s="63"/>
+      <c r="G48" s="63"/>
+      <c r="H48" s="63"/>
+      <c r="I48" s="63"/>
+      <c r="J48" s="63"/>
+      <c r="K48" s="63"/>
+      <c r="L48" s="64"/>
+    </row>
+    <row r="49" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A49" s="62"/>
+      <c r="B49" s="63"/>
+      <c r="C49" s="63"/>
+      <c r="D49" s="63"/>
+      <c r="E49" s="63"/>
+      <c r="F49" s="63"/>
+      <c r="G49" s="63"/>
+      <c r="H49" s="63"/>
+      <c r="I49" s="63"/>
+      <c r="J49" s="63"/>
+      <c r="K49" s="63"/>
+      <c r="L49" s="64"/>
+    </row>
+    <row r="50" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A50" s="62"/>
+      <c r="B50" s="63"/>
+      <c r="C50" s="63"/>
+      <c r="D50" s="63"/>
+      <c r="E50" s="63"/>
+      <c r="F50" s="63"/>
+      <c r="G50" s="63"/>
+      <c r="H50" s="63"/>
+      <c r="I50" s="63"/>
+      <c r="J50" s="63"/>
+      <c r="K50" s="63"/>
+      <c r="L50" s="64"/>
+    </row>
+    <row r="51" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A51" s="62"/>
+      <c r="B51" s="63"/>
+      <c r="C51" s="63"/>
+      <c r="D51" s="63"/>
+      <c r="E51" s="63"/>
+      <c r="F51" s="63"/>
+      <c r="G51" s="63"/>
+      <c r="H51" s="63"/>
+      <c r="I51" s="63"/>
+      <c r="J51" s="63"/>
+      <c r="K51" s="63"/>
+      <c r="L51" s="64"/>
+    </row>
+    <row r="52" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A52" s="62"/>
+      <c r="B52" s="63"/>
+      <c r="C52" s="63"/>
+      <c r="D52" s="63"/>
+      <c r="E52" s="63"/>
+      <c r="F52" s="63"/>
+      <c r="G52" s="63"/>
+      <c r="H52" s="63"/>
+      <c r="I52" s="63"/>
+      <c r="J52" s="63"/>
+      <c r="K52" s="63"/>
+      <c r="L52" s="64"/>
+    </row>
+    <row r="53" spans="1:12" ht="25.2" customHeight="1">
+      <c r="A53" s="65"/>
+      <c r="B53" s="66"/>
+      <c r="C53" s="66"/>
+      <c r="D53" s="66"/>
+      <c r="E53" s="66"/>
+      <c r="F53" s="66"/>
+      <c r="G53" s="66"/>
+      <c r="H53" s="66"/>
+      <c r="I53" s="66"/>
+      <c r="J53" s="66"/>
+      <c r="K53" s="66"/>
+      <c r="L53" s="67"/>
+    </row>
+    <row r="55" spans="1:12" ht="16.8">
+      <c r="A55" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="B45" s="56"/>
-      <c r="C45" s="56"/>
-      <c r="D45" s="56"/>
-      <c r="E45" s="56"/>
-      <c r="F45" s="56"/>
-      <c r="G45" s="56"/>
-      <c r="H45" s="56"/>
-      <c r="I45" s="56"/>
-      <c r="J45" s="56"/>
-      <c r="K45" s="56"/>
-      <c r="L45" s="57"/>
-    </row>
-    <row r="46" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A46" s="58" t="s">
+      <c r="B55" s="57"/>
+      <c r="C55" s="57"/>
+      <c r="D55" s="57"/>
+      <c r="E55" s="57"/>
+      <c r="F55" s="57"/>
+      <c r="G55" s="57"/>
+      <c r="H55" s="57"/>
+      <c r="I55" s="57"/>
+      <c r="J55" s="57"/>
+      <c r="K55" s="57"/>
+      <c r="L55" s="58"/>
+    </row>
+    <row r="56" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A56" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="B46" s="59"/>
-      <c r="C46" s="59"/>
-      <c r="D46" s="59"/>
-      <c r="E46" s="59"/>
-      <c r="F46" s="59"/>
-      <c r="G46" s="59"/>
-      <c r="H46" s="59"/>
-      <c r="I46" s="59"/>
-      <c r="J46" s="59"/>
-      <c r="K46" s="59"/>
-      <c r="L46" s="60"/>
-    </row>
-    <row r="47" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A47" s="61"/>
-      <c r="B47" s="62"/>
-      <c r="C47" s="62"/>
-      <c r="D47" s="62"/>
-      <c r="E47" s="62"/>
-      <c r="F47" s="62"/>
-      <c r="G47" s="62"/>
-      <c r="H47" s="62"/>
-      <c r="I47" s="62"/>
-      <c r="J47" s="62"/>
-      <c r="K47" s="62"/>
-      <c r="L47" s="63"/>
-    </row>
-    <row r="48" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A48" s="61"/>
-      <c r="B48" s="62"/>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="62"/>
-      <c r="L48" s="63"/>
-    </row>
-    <row r="49" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A49" s="61"/>
-      <c r="B49" s="62"/>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="62"/>
-      <c r="L49" s="63"/>
-    </row>
-    <row r="50" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A50" s="61"/>
-      <c r="B50" s="62"/>
-      <c r="C50" s="62"/>
-      <c r="D50" s="62"/>
-      <c r="E50" s="62"/>
-      <c r="F50" s="62"/>
-      <c r="G50" s="62"/>
-      <c r="H50" s="62"/>
-      <c r="I50" s="62"/>
-      <c r="J50" s="62"/>
-      <c r="K50" s="62"/>
-      <c r="L50" s="63"/>
-    </row>
-    <row r="51" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A51" s="61"/>
-      <c r="B51" s="62"/>
-      <c r="C51" s="62"/>
-      <c r="D51" s="62"/>
-      <c r="E51" s="62"/>
-      <c r="F51" s="62"/>
-      <c r="G51" s="62"/>
-      <c r="H51" s="62"/>
-      <c r="I51" s="62"/>
-      <c r="J51" s="62"/>
-      <c r="K51" s="62"/>
-      <c r="L51" s="63"/>
-    </row>
-    <row r="52" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A52" s="61"/>
-      <c r="B52" s="62"/>
-      <c r="C52" s="62"/>
-      <c r="D52" s="62"/>
-      <c r="E52" s="62"/>
-      <c r="F52" s="62"/>
-      <c r="G52" s="62"/>
-      <c r="H52" s="62"/>
-      <c r="I52" s="62"/>
-      <c r="J52" s="62"/>
-      <c r="K52" s="62"/>
-      <c r="L52" s="63"/>
-    </row>
-    <row r="53" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A53" s="64"/>
-      <c r="B53" s="65"/>
-      <c r="C53" s="65"/>
-      <c r="D53" s="65"/>
-      <c r="E53" s="65"/>
-      <c r="F53" s="65"/>
-      <c r="G53" s="65"/>
-      <c r="H53" s="65"/>
-      <c r="I53" s="65"/>
-      <c r="J53" s="65"/>
-      <c r="K53" s="65"/>
-      <c r="L53" s="66"/>
-    </row>
-    <row r="55" spans="1:12" ht="16.8">
-      <c r="A55" s="55" t="s">
+      <c r="B56" s="60"/>
+      <c r="C56" s="60"/>
+      <c r="D56" s="60"/>
+      <c r="E56" s="60"/>
+      <c r="F56" s="60"/>
+      <c r="G56" s="60"/>
+      <c r="H56" s="60"/>
+      <c r="I56" s="60"/>
+      <c r="J56" s="60"/>
+      <c r="K56" s="60"/>
+      <c r="L56" s="61"/>
+    </row>
+    <row r="57" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A57" s="62"/>
+      <c r="B57" s="63"/>
+      <c r="C57" s="63"/>
+      <c r="D57" s="63"/>
+      <c r="E57" s="63"/>
+      <c r="F57" s="63"/>
+      <c r="G57" s="63"/>
+      <c r="H57" s="63"/>
+      <c r="I57" s="63"/>
+      <c r="J57" s="63"/>
+      <c r="K57" s="63"/>
+      <c r="L57" s="64"/>
+    </row>
+    <row r="58" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A58" s="62"/>
+      <c r="B58" s="63"/>
+      <c r="C58" s="63"/>
+      <c r="D58" s="63"/>
+      <c r="E58" s="63"/>
+      <c r="F58" s="63"/>
+      <c r="G58" s="63"/>
+      <c r="H58" s="63"/>
+      <c r="I58" s="63"/>
+      <c r="J58" s="63"/>
+      <c r="K58" s="63"/>
+      <c r="L58" s="64"/>
+    </row>
+    <row r="59" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A59" s="62"/>
+      <c r="B59" s="63"/>
+      <c r="C59" s="63"/>
+      <c r="D59" s="63"/>
+      <c r="E59" s="63"/>
+      <c r="F59" s="63"/>
+      <c r="G59" s="63"/>
+      <c r="H59" s="63"/>
+      <c r="I59" s="63"/>
+      <c r="J59" s="63"/>
+      <c r="K59" s="63"/>
+      <c r="L59" s="64"/>
+    </row>
+    <row r="60" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A60" s="62"/>
+      <c r="B60" s="63"/>
+      <c r="C60" s="63"/>
+      <c r="D60" s="63"/>
+      <c r="E60" s="63"/>
+      <c r="F60" s="63"/>
+      <c r="G60" s="63"/>
+      <c r="H60" s="63"/>
+      <c r="I60" s="63"/>
+      <c r="J60" s="63"/>
+      <c r="K60" s="63"/>
+      <c r="L60" s="64"/>
+    </row>
+    <row r="61" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A61" s="62"/>
+      <c r="B61" s="63"/>
+      <c r="C61" s="63"/>
+      <c r="D61" s="63"/>
+      <c r="E61" s="63"/>
+      <c r="F61" s="63"/>
+      <c r="G61" s="63"/>
+      <c r="H61" s="63"/>
+      <c r="I61" s="63"/>
+      <c r="J61" s="63"/>
+      <c r="K61" s="63"/>
+      <c r="L61" s="64"/>
+    </row>
+    <row r="62" spans="1:12" ht="7.2" customHeight="1">
+      <c r="A62" s="62"/>
+      <c r="B62" s="63"/>
+      <c r="C62" s="63"/>
+      <c r="D62" s="63"/>
+      <c r="E62" s="63"/>
+      <c r="F62" s="63"/>
+      <c r="G62" s="63"/>
+      <c r="H62" s="63"/>
+      <c r="I62" s="63"/>
+      <c r="J62" s="63"/>
+      <c r="K62" s="63"/>
+      <c r="L62" s="64"/>
+    </row>
+    <row r="63" spans="1:12" ht="18" hidden="1" customHeight="1">
+      <c r="A63" s="62"/>
+      <c r="B63" s="63"/>
+      <c r="C63" s="63"/>
+      <c r="D63" s="63"/>
+      <c r="E63" s="63"/>
+      <c r="F63" s="63"/>
+      <c r="G63" s="63"/>
+      <c r="H63" s="63"/>
+      <c r="I63" s="63"/>
+      <c r="J63" s="63"/>
+      <c r="K63" s="63"/>
+      <c r="L63" s="64"/>
+    </row>
+    <row r="64" spans="1:12" ht="18" hidden="1" customHeight="1">
+      <c r="A64" s="65"/>
+      <c r="B64" s="66"/>
+      <c r="C64" s="66"/>
+      <c r="D64" s="66"/>
+      <c r="E64" s="66"/>
+      <c r="F64" s="66"/>
+      <c r="G64" s="66"/>
+      <c r="H64" s="66"/>
+      <c r="I64" s="66"/>
+      <c r="J64" s="66"/>
+      <c r="K64" s="66"/>
+      <c r="L64" s="67"/>
+    </row>
+    <row r="66" spans="1:12" ht="7.2" customHeight="1">
+      <c r="A66" s="69"/>
+      <c r="B66" s="69"/>
+      <c r="C66" s="69"/>
+      <c r="D66" s="69"/>
+      <c r="E66" s="69"/>
+      <c r="F66" s="69"/>
+      <c r="G66" s="69"/>
+      <c r="H66" s="69"/>
+      <c r="I66" s="69"/>
+      <c r="J66" s="69"/>
+      <c r="K66" s="69"/>
+      <c r="L66" s="69"/>
+    </row>
+    <row r="67" spans="1:12" hidden="1">
+      <c r="A67" s="69"/>
+      <c r="B67" s="69"/>
+      <c r="C67" s="69"/>
+      <c r="D67" s="69"/>
+      <c r="E67" s="69"/>
+      <c r="F67" s="69"/>
+      <c r="G67" s="69"/>
+      <c r="H67" s="69"/>
+      <c r="I67" s="69"/>
+      <c r="J67" s="69"/>
+      <c r="K67" s="69"/>
+      <c r="L67" s="69"/>
+    </row>
+    <row r="69" spans="1:12" ht="17.399999999999999">
+      <c r="A69" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="B55" s="56"/>
-      <c r="C55" s="56"/>
-      <c r="D55" s="56"/>
-      <c r="E55" s="56"/>
-      <c r="F55" s="56"/>
-      <c r="G55" s="56"/>
-      <c r="H55" s="56"/>
-      <c r="I55" s="56"/>
-      <c r="J55" s="56"/>
-      <c r="K55" s="56"/>
-      <c r="L55" s="57"/>
-    </row>
-    <row r="56" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A56" s="58" t="s">
+      <c r="B69" s="71"/>
+      <c r="C69" s="71"/>
+      <c r="D69" s="71"/>
+      <c r="E69" s="71"/>
+      <c r="F69" s="71"/>
+      <c r="G69" s="71"/>
+      <c r="H69" s="71"/>
+      <c r="I69" s="71"/>
+      <c r="J69" s="71"/>
+      <c r="K69" s="71"/>
+      <c r="L69" s="72"/>
+    </row>
+    <row r="70" spans="1:12">
+      <c r="A70" s="73" t="s">
         <v>16</v>
       </c>
-      <c r="B56" s="59"/>
-      <c r="C56" s="59"/>
-      <c r="D56" s="59"/>
-      <c r="E56" s="59"/>
-      <c r="F56" s="59"/>
-      <c r="G56" s="59"/>
-      <c r="H56" s="59"/>
-      <c r="I56" s="59"/>
-      <c r="J56" s="59"/>
-      <c r="K56" s="59"/>
-      <c r="L56" s="60"/>
-    </row>
-    <row r="57" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A57" s="61"/>
-      <c r="B57" s="62"/>
-      <c r="C57" s="62"/>
-      <c r="D57" s="62"/>
-      <c r="E57" s="62"/>
-      <c r="F57" s="62"/>
-      <c r="G57" s="62"/>
-      <c r="H57" s="62"/>
-      <c r="I57" s="62"/>
-      <c r="J57" s="62"/>
-      <c r="K57" s="62"/>
-      <c r="L57" s="63"/>
-    </row>
-    <row r="58" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A58" s="61"/>
-      <c r="B58" s="62"/>
-      <c r="C58" s="62"/>
-      <c r="D58" s="62"/>
-      <c r="E58" s="62"/>
-      <c r="F58" s="62"/>
-      <c r="G58" s="62"/>
-      <c r="H58" s="62"/>
-      <c r="I58" s="62"/>
-      <c r="J58" s="62"/>
-      <c r="K58" s="62"/>
-      <c r="L58" s="63"/>
-    </row>
-    <row r="59" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A59" s="61"/>
-      <c r="B59" s="62"/>
-      <c r="C59" s="62"/>
-      <c r="D59" s="62"/>
-      <c r="E59" s="62"/>
-      <c r="F59" s="62"/>
-      <c r="G59" s="62"/>
-      <c r="H59" s="62"/>
-      <c r="I59" s="62"/>
-      <c r="J59" s="62"/>
-      <c r="K59" s="62"/>
-      <c r="L59" s="63"/>
-    </row>
-    <row r="60" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A60" s="61"/>
-      <c r="B60" s="62"/>
-      <c r="C60" s="62"/>
-      <c r="D60" s="62"/>
-      <c r="E60" s="62"/>
-      <c r="F60" s="62"/>
-      <c r="G60" s="62"/>
-      <c r="H60" s="62"/>
-      <c r="I60" s="62"/>
-      <c r="J60" s="62"/>
-      <c r="K60" s="62"/>
-      <c r="L60" s="63"/>
-    </row>
-    <row r="61" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A61" s="61"/>
-      <c r="B61" s="62"/>
-      <c r="C61" s="62"/>
-      <c r="D61" s="62"/>
-      <c r="E61" s="62"/>
-      <c r="F61" s="62"/>
-      <c r="G61" s="62"/>
-      <c r="H61" s="62"/>
-      <c r="I61" s="62"/>
-      <c r="J61" s="62"/>
-      <c r="K61" s="62"/>
-      <c r="L61" s="63"/>
-    </row>
-    <row r="62" spans="1:12" ht="7.2" customHeight="1">
-      <c r="A62" s="61"/>
-      <c r="B62" s="62"/>
-      <c r="C62" s="62"/>
-      <c r="D62" s="62"/>
-      <c r="E62" s="62"/>
-      <c r="F62" s="62"/>
-      <c r="G62" s="62"/>
-      <c r="H62" s="62"/>
-      <c r="I62" s="62"/>
-      <c r="J62" s="62"/>
-      <c r="K62" s="62"/>
-      <c r="L62" s="63"/>
-    </row>
-    <row r="63" spans="1:12" ht="18" hidden="1" customHeight="1">
-      <c r="A63" s="61"/>
-      <c r="B63" s="62"/>
-      <c r="C63" s="62"/>
-      <c r="D63" s="62"/>
-      <c r="E63" s="62"/>
-      <c r="F63" s="62"/>
-      <c r="G63" s="62"/>
-      <c r="H63" s="62"/>
-      <c r="I63" s="62"/>
-      <c r="J63" s="62"/>
-      <c r="K63" s="62"/>
-      <c r="L63" s="63"/>
-    </row>
-    <row r="64" spans="1:12" ht="18" hidden="1" customHeight="1">
-      <c r="A64" s="64"/>
-      <c r="B64" s="65"/>
-      <c r="C64" s="65"/>
-      <c r="D64" s="65"/>
-      <c r="E64" s="65"/>
-      <c r="F64" s="65"/>
-      <c r="G64" s="65"/>
-      <c r="H64" s="65"/>
-      <c r="I64" s="65"/>
-      <c r="J64" s="65"/>
-      <c r="K64" s="65"/>
-      <c r="L64" s="66"/>
-    </row>
-    <row r="66" spans="1:12" ht="7.2" customHeight="1">
-      <c r="A66" s="67"/>
-      <c r="B66" s="67"/>
-      <c r="C66" s="67"/>
-      <c r="D66" s="67"/>
-      <c r="E66" s="67"/>
-      <c r="F66" s="67"/>
-      <c r="G66" s="67"/>
-      <c r="H66" s="67"/>
-      <c r="I66" s="67"/>
-      <c r="J66" s="67"/>
-      <c r="K66" s="67"/>
-      <c r="L66" s="67"/>
-    </row>
-    <row r="67" spans="1:12" hidden="1">
-      <c r="A67" s="67"/>
-      <c r="B67" s="67"/>
-      <c r="C67" s="67"/>
-      <c r="D67" s="67"/>
-      <c r="E67" s="67"/>
-      <c r="F67" s="67"/>
-      <c r="G67" s="67"/>
-      <c r="H67" s="67"/>
-      <c r="I67" s="67"/>
-      <c r="J67" s="67"/>
-      <c r="K67" s="67"/>
-      <c r="L67" s="67"/>
-    </row>
-    <row r="69" spans="1:12" ht="17.399999999999999">
-      <c r="A69" s="68" t="s">
+      <c r="B70" s="74"/>
+      <c r="C70" s="74"/>
+      <c r="D70" s="74"/>
+      <c r="E70" s="74"/>
+      <c r="F70" s="74"/>
+      <c r="G70" s="74"/>
+      <c r="H70" s="74"/>
+      <c r="I70" s="74"/>
+      <c r="J70" s="74"/>
+      <c r="K70" s="74"/>
+      <c r="L70" s="75"/>
+    </row>
+    <row r="71" spans="1:12">
+      <c r="A71" s="76"/>
+      <c r="B71" s="77"/>
+      <c r="C71" s="77"/>
+      <c r="D71" s="77"/>
+      <c r="E71" s="77"/>
+      <c r="F71" s="77"/>
+      <c r="G71" s="77"/>
+      <c r="H71" s="77"/>
+      <c r="I71" s="77"/>
+      <c r="J71" s="77"/>
+      <c r="K71" s="77"/>
+      <c r="L71" s="78"/>
+    </row>
+    <row r="72" spans="1:12">
+      <c r="A72" s="79"/>
+      <c r="B72" s="80"/>
+      <c r="C72" s="80"/>
+      <c r="D72" s="80"/>
+      <c r="E72" s="80"/>
+      <c r="F72" s="80"/>
+      <c r="G72" s="80"/>
+      <c r="H72" s="80"/>
+      <c r="I72" s="80"/>
+      <c r="J72" s="80"/>
+      <c r="K72" s="80"/>
+      <c r="L72" s="81"/>
+    </row>
+    <row r="74" spans="1:12" ht="15.6">
+      <c r="A74" s="82" t="s">
         <v>17</v>
       </c>
-      <c r="B69" s="69"/>
-      <c r="C69" s="69"/>
-      <c r="D69" s="69"/>
-      <c r="E69" s="69"/>
-      <c r="F69" s="69"/>
-      <c r="G69" s="69"/>
-      <c r="H69" s="69"/>
-      <c r="I69" s="69"/>
-      <c r="J69" s="69"/>
-      <c r="K69" s="69"/>
-      <c r="L69" s="70"/>
-    </row>
-    <row r="70" spans="1:12">
-      <c r="A70" s="71" t="s">
+      <c r="B74" s="83"/>
+      <c r="C74" s="83"/>
+      <c r="D74" s="83"/>
+      <c r="E74" s="83"/>
+      <c r="F74" s="83"/>
+      <c r="G74" s="83"/>
+      <c r="H74" s="83"/>
+      <c r="I74" s="83"/>
+      <c r="J74" s="83"/>
+      <c r="K74" s="83"/>
+      <c r="L74" s="84"/>
+    </row>
+    <row r="75" spans="1:12" ht="24" customHeight="1">
+      <c r="A75" s="85" t="s">
         <v>18</v>
       </c>
-      <c r="B70" s="72"/>
-      <c r="C70" s="72"/>
-      <c r="D70" s="72"/>
-      <c r="E70" s="72"/>
-      <c r="F70" s="72"/>
-      <c r="G70" s="72"/>
-      <c r="H70" s="72"/>
-      <c r="I70" s="72"/>
-      <c r="J70" s="72"/>
-      <c r="K70" s="72"/>
-      <c r="L70" s="73"/>
-    </row>
-    <row r="71" spans="1:12">
-      <c r="A71" s="74"/>
-      <c r="B71" s="75"/>
-      <c r="C71" s="75"/>
-      <c r="D71" s="75"/>
-      <c r="E71" s="75"/>
-      <c r="F71" s="75"/>
-      <c r="G71" s="75"/>
-      <c r="H71" s="75"/>
-      <c r="I71" s="75"/>
-      <c r="J71" s="75"/>
-      <c r="K71" s="75"/>
-      <c r="L71" s="76"/>
-    </row>
-    <row r="72" spans="1:12">
-      <c r="A72" s="77"/>
-      <c r="B72" s="78"/>
-      <c r="C72" s="78"/>
-      <c r="D72" s="78"/>
-      <c r="E72" s="78"/>
-      <c r="F72" s="78"/>
-      <c r="G72" s="78"/>
-      <c r="H72" s="78"/>
-      <c r="I72" s="78"/>
-      <c r="J72" s="78"/>
-      <c r="K72" s="78"/>
-      <c r="L72" s="79"/>
-    </row>
-    <row r="74" spans="1:12" ht="15.6">
-      <c r="A74" s="80" t="s">
+      <c r="B75" s="86"/>
+      <c r="C75" s="86"/>
+      <c r="D75" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="B74" s="81"/>
-      <c r="C74" s="81"/>
-      <c r="D74" s="81"/>
-      <c r="E74" s="81"/>
-      <c r="F74" s="81"/>
-      <c r="G74" s="81"/>
-      <c r="H74" s="81"/>
-      <c r="I74" s="81"/>
-      <c r="J74" s="81"/>
-      <c r="K74" s="81"/>
-      <c r="L74" s="82"/>
-    </row>
-    <row r="75" spans="1:12" ht="24" customHeight="1">
-      <c r="A75" s="83" t="s">
+      <c r="E75" s="86"/>
+      <c r="F75" s="86"/>
+      <c r="G75" s="86"/>
+      <c r="H75" s="86"/>
+      <c r="I75" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="B75" s="84"/>
-      <c r="C75" s="84"/>
-      <c r="D75" s="84" t="s">
+      <c r="J75" s="86"/>
+      <c r="K75" s="86"/>
+      <c r="L75" s="87"/>
+    </row>
+    <row r="76" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A76" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="E75" s="84"/>
-      <c r="F75" s="84"/>
-      <c r="G75" s="84"/>
-      <c r="H75" s="84"/>
-      <c r="I75" s="84" t="s">
+      <c r="B76" s="89"/>
+      <c r="C76" s="89"/>
+      <c r="D76" s="94" t="s">
         <v>22</v>
       </c>
-      <c r="J75" s="84"/>
-      <c r="K75" s="84"/>
-      <c r="L75" s="85"/>
-    </row>
-    <row r="76" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A76" s="86" t="s">
+      <c r="E76" s="94"/>
+      <c r="F76" s="94"/>
+      <c r="G76" s="94"/>
+      <c r="H76" s="94"/>
+      <c r="I76" s="94" t="s">
         <v>23</v>
       </c>
-      <c r="B76" s="87"/>
-      <c r="C76" s="87"/>
-      <c r="D76" s="92" t="s">
+      <c r="J76" s="94"/>
+      <c r="K76" s="94"/>
+      <c r="L76" s="97"/>
+    </row>
+    <row r="77" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A77" s="90"/>
+      <c r="B77" s="91"/>
+      <c r="C77" s="91"/>
+      <c r="D77" s="95"/>
+      <c r="E77" s="95"/>
+      <c r="F77" s="95"/>
+      <c r="G77" s="95"/>
+      <c r="H77" s="95"/>
+      <c r="I77" s="95"/>
+      <c r="J77" s="95"/>
+      <c r="K77" s="95"/>
+      <c r="L77" s="98"/>
+    </row>
+    <row r="78" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A78" s="90"/>
+      <c r="B78" s="91"/>
+      <c r="C78" s="91"/>
+      <c r="D78" s="95"/>
+      <c r="E78" s="95"/>
+      <c r="F78" s="95"/>
+      <c r="G78" s="95"/>
+      <c r="H78" s="95"/>
+      <c r="I78" s="95"/>
+      <c r="J78" s="95"/>
+      <c r="K78" s="95"/>
+      <c r="L78" s="98"/>
+    </row>
+    <row r="79" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A79" s="92"/>
+      <c r="B79" s="93"/>
+      <c r="C79" s="93"/>
+      <c r="D79" s="96"/>
+      <c r="E79" s="96"/>
+      <c r="F79" s="96"/>
+      <c r="G79" s="96"/>
+      <c r="H79" s="96"/>
+      <c r="I79" s="96"/>
+      <c r="J79" s="96"/>
+      <c r="K79" s="96"/>
+      <c r="L79" s="99"/>
+    </row>
+    <row r="80" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A80" s="100" t="s">
         <v>24</v>
       </c>
-      <c r="E76" s="92"/>
-      <c r="F76" s="92"/>
-      <c r="G76" s="92"/>
-      <c r="H76" s="92"/>
-      <c r="I76" s="92" t="s">
+      <c r="B80" s="101"/>
+      <c r="C80" s="101"/>
+      <c r="D80" s="106" t="s">
         <v>25</v>
       </c>
-      <c r="J76" s="92"/>
-      <c r="K76" s="92"/>
-      <c r="L76" s="95"/>
-    </row>
-    <row r="77" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A77" s="88"/>
-      <c r="B77" s="89"/>
-      <c r="C77" s="89"/>
-      <c r="D77" s="93"/>
-      <c r="E77" s="93"/>
-      <c r="F77" s="93"/>
-      <c r="G77" s="93"/>
-      <c r="H77" s="93"/>
-      <c r="I77" s="93"/>
-      <c r="J77" s="93"/>
-      <c r="K77" s="93"/>
-      <c r="L77" s="96"/>
-    </row>
-    <row r="78" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A78" s="88"/>
-      <c r="B78" s="89"/>
-      <c r="C78" s="89"/>
-      <c r="D78" s="93"/>
-      <c r="E78" s="93"/>
-      <c r="F78" s="93"/>
-      <c r="G78" s="93"/>
-      <c r="H78" s="93"/>
-      <c r="I78" s="93"/>
-      <c r="J78" s="93"/>
-      <c r="K78" s="93"/>
-      <c r="L78" s="96"/>
-    </row>
-    <row r="79" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A79" s="90"/>
-      <c r="B79" s="91"/>
-      <c r="C79" s="91"/>
-      <c r="D79" s="94"/>
-      <c r="E79" s="94"/>
-      <c r="F79" s="94"/>
-      <c r="G79" s="94"/>
-      <c r="H79" s="94"/>
-      <c r="I79" s="94"/>
-      <c r="J79" s="94"/>
-      <c r="K79" s="94"/>
-      <c r="L79" s="97"/>
-    </row>
-    <row r="80" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A80" s="98" t="s">
+      <c r="E80" s="106"/>
+      <c r="F80" s="106"/>
+      <c r="G80" s="106"/>
+      <c r="H80" s="106"/>
+      <c r="I80" s="106" t="s">
         <v>26</v>
       </c>
-      <c r="B80" s="99"/>
-      <c r="C80" s="99"/>
-      <c r="D80" s="104" t="s">
+      <c r="J80" s="106"/>
+      <c r="K80" s="106"/>
+      <c r="L80" s="109"/>
+    </row>
+    <row r="81" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A81" s="102"/>
+      <c r="B81" s="103"/>
+      <c r="C81" s="103"/>
+      <c r="D81" s="107"/>
+      <c r="E81" s="107"/>
+      <c r="F81" s="107"/>
+      <c r="G81" s="107"/>
+      <c r="H81" s="107"/>
+      <c r="I81" s="107"/>
+      <c r="J81" s="107"/>
+      <c r="K81" s="107"/>
+      <c r="L81" s="110"/>
+    </row>
+    <row r="82" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A82" s="102"/>
+      <c r="B82" s="103"/>
+      <c r="C82" s="103"/>
+      <c r="D82" s="107"/>
+      <c r="E82" s="107"/>
+      <c r="F82" s="107"/>
+      <c r="G82" s="107"/>
+      <c r="H82" s="107"/>
+      <c r="I82" s="107"/>
+      <c r="J82" s="107"/>
+      <c r="K82" s="107"/>
+      <c r="L82" s="110"/>
+    </row>
+    <row r="83" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A83" s="104"/>
+      <c r="B83" s="105"/>
+      <c r="C83" s="105"/>
+      <c r="D83" s="108"/>
+      <c r="E83" s="108"/>
+      <c r="F83" s="108"/>
+      <c r="G83" s="108"/>
+      <c r="H83" s="108"/>
+      <c r="I83" s="108"/>
+      <c r="J83" s="108"/>
+      <c r="K83" s="108"/>
+      <c r="L83" s="111"/>
+    </row>
+    <row r="84" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A84" s="88" t="s">
         <v>27</v>
       </c>
-      <c r="E80" s="104"/>
-      <c r="F80" s="104"/>
-      <c r="G80" s="104"/>
-      <c r="H80" s="104"/>
-      <c r="I80" s="104" t="s">
+      <c r="B84" s="89"/>
+      <c r="C84" s="89"/>
+      <c r="D84" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="J80" s="104"/>
-      <c r="K80" s="104"/>
-      <c r="L80" s="107"/>
-    </row>
-    <row r="81" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A81" s="100"/>
-      <c r="B81" s="101"/>
-      <c r="C81" s="101"/>
-      <c r="D81" s="105"/>
-      <c r="E81" s="105"/>
-      <c r="F81" s="105"/>
-      <c r="G81" s="105"/>
-      <c r="H81" s="105"/>
-      <c r="I81" s="105"/>
-      <c r="J81" s="105"/>
-      <c r="K81" s="105"/>
-      <c r="L81" s="108"/>
-    </row>
-    <row r="82" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A82" s="100"/>
-      <c r="B82" s="101"/>
-      <c r="C82" s="101"/>
-      <c r="D82" s="105"/>
-      <c r="E82" s="105"/>
-      <c r="F82" s="105"/>
-      <c r="G82" s="105"/>
-      <c r="H82" s="105"/>
-      <c r="I82" s="105"/>
-      <c r="J82" s="105"/>
-      <c r="K82" s="105"/>
-      <c r="L82" s="108"/>
-    </row>
-    <row r="83" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A83" s="102"/>
-      <c r="B83" s="103"/>
-      <c r="C83" s="103"/>
-      <c r="D83" s="106"/>
-      <c r="E83" s="106"/>
-      <c r="F83" s="106"/>
-      <c r="G83" s="106"/>
-      <c r="H83" s="106"/>
-      <c r="I83" s="106"/>
-      <c r="J83" s="106"/>
-      <c r="K83" s="106"/>
-      <c r="L83" s="109"/>
-    </row>
-    <row r="84" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A84" s="86" t="s">
+      <c r="E84" s="94"/>
+      <c r="F84" s="94"/>
+      <c r="G84" s="94"/>
+      <c r="H84" s="94"/>
+      <c r="I84" s="94" t="s">
         <v>29</v>
       </c>
-      <c r="B84" s="87"/>
-      <c r="C84" s="87"/>
-      <c r="D84" s="92" t="s">
+      <c r="J84" s="94"/>
+      <c r="K84" s="94"/>
+      <c r="L84" s="97"/>
+    </row>
+    <row r="85" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A85" s="90"/>
+      <c r="B85" s="91"/>
+      <c r="C85" s="91"/>
+      <c r="D85" s="95"/>
+      <c r="E85" s="95"/>
+      <c r="F85" s="95"/>
+      <c r="G85" s="95"/>
+      <c r="H85" s="95"/>
+      <c r="I85" s="95"/>
+      <c r="J85" s="95"/>
+      <c r="K85" s="95"/>
+      <c r="L85" s="98"/>
+    </row>
+    <row r="86" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A86" s="90"/>
+      <c r="B86" s="91"/>
+      <c r="C86" s="91"/>
+      <c r="D86" s="95"/>
+      <c r="E86" s="95"/>
+      <c r="F86" s="95"/>
+      <c r="G86" s="95"/>
+      <c r="H86" s="95"/>
+      <c r="I86" s="95"/>
+      <c r="J86" s="95"/>
+      <c r="K86" s="95"/>
+      <c r="L86" s="98"/>
+    </row>
+    <row r="87" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A87" s="92"/>
+      <c r="B87" s="93"/>
+      <c r="C87" s="93"/>
+      <c r="D87" s="96"/>
+      <c r="E87" s="96"/>
+      <c r="F87" s="96"/>
+      <c r="G87" s="96"/>
+      <c r="H87" s="96"/>
+      <c r="I87" s="96"/>
+      <c r="J87" s="96"/>
+      <c r="K87" s="96"/>
+      <c r="L87" s="99"/>
+    </row>
+    <row r="88" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A88" s="100" t="s">
         <v>30</v>
       </c>
-      <c r="E84" s="92"/>
-      <c r="F84" s="92"/>
-      <c r="G84" s="92"/>
-      <c r="H84" s="92"/>
-      <c r="I84" s="92" t="s">
+      <c r="B88" s="101"/>
+      <c r="C88" s="101"/>
+      <c r="D88" s="106" t="s">
         <v>31</v>
       </c>
-      <c r="J84" s="92"/>
-      <c r="K84" s="92"/>
-      <c r="L84" s="95"/>
-    </row>
-    <row r="85" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A85" s="88"/>
-      <c r="B85" s="89"/>
-      <c r="C85" s="89"/>
-      <c r="D85" s="93"/>
-      <c r="E85" s="93"/>
-      <c r="F85" s="93"/>
-      <c r="G85" s="93"/>
-      <c r="H85" s="93"/>
-      <c r="I85" s="93"/>
-      <c r="J85" s="93"/>
-      <c r="K85" s="93"/>
-      <c r="L85" s="96"/>
-    </row>
-    <row r="86" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A86" s="88"/>
-      <c r="B86" s="89"/>
-      <c r="C86" s="89"/>
-      <c r="D86" s="93"/>
-      <c r="E86" s="93"/>
-      <c r="F86" s="93"/>
-      <c r="G86" s="93"/>
-      <c r="H86" s="93"/>
-      <c r="I86" s="93"/>
-      <c r="J86" s="93"/>
-      <c r="K86" s="93"/>
-      <c r="L86" s="96"/>
-    </row>
-    <row r="87" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A87" s="90"/>
-      <c r="B87" s="91"/>
-      <c r="C87" s="91"/>
-      <c r="D87" s="94"/>
-      <c r="E87" s="94"/>
-      <c r="F87" s="94"/>
-      <c r="G87" s="94"/>
-      <c r="H87" s="94"/>
-      <c r="I87" s="94"/>
-      <c r="J87" s="94"/>
-      <c r="K87" s="94"/>
-      <c r="L87" s="97"/>
-    </row>
-    <row r="88" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A88" s="98" t="s">
+      <c r="E88" s="106"/>
+      <c r="F88" s="106"/>
+      <c r="G88" s="106"/>
+      <c r="H88" s="106"/>
+      <c r="I88" s="106" t="s">
         <v>32</v>
       </c>
-      <c r="B88" s="99"/>
-      <c r="C88" s="99"/>
-      <c r="D88" s="104" t="s">
+      <c r="J88" s="106"/>
+      <c r="K88" s="106"/>
+      <c r="L88" s="109"/>
+    </row>
+    <row r="89" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A89" s="102"/>
+      <c r="B89" s="103"/>
+      <c r="C89" s="103"/>
+      <c r="D89" s="107"/>
+      <c r="E89" s="107"/>
+      <c r="F89" s="107"/>
+      <c r="G89" s="107"/>
+      <c r="H89" s="107"/>
+      <c r="I89" s="107"/>
+      <c r="J89" s="107"/>
+      <c r="K89" s="107"/>
+      <c r="L89" s="110"/>
+    </row>
+    <row r="90" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A90" s="102"/>
+      <c r="B90" s="103"/>
+      <c r="C90" s="103"/>
+      <c r="D90" s="107"/>
+      <c r="E90" s="107"/>
+      <c r="F90" s="107"/>
+      <c r="G90" s="107"/>
+      <c r="H90" s="107"/>
+      <c r="I90" s="107"/>
+      <c r="J90" s="107"/>
+      <c r="K90" s="107"/>
+      <c r="L90" s="110"/>
+    </row>
+    <row r="91" spans="1:12" ht="19.2" customHeight="1">
+      <c r="A91" s="104"/>
+      <c r="B91" s="105"/>
+      <c r="C91" s="105"/>
+      <c r="D91" s="108"/>
+      <c r="E91" s="108"/>
+      <c r="F91" s="108"/>
+      <c r="G91" s="108"/>
+      <c r="H91" s="108"/>
+      <c r="I91" s="108"/>
+      <c r="J91" s="108"/>
+      <c r="K91" s="108"/>
+      <c r="L91" s="111"/>
+    </row>
+    <row r="93" spans="1:12" ht="15.6">
+      <c r="A93" s="112" t="s">
         <v>33</v>
       </c>
-      <c r="E88" s="104"/>
-      <c r="F88" s="104"/>
-      <c r="G88" s="104"/>
-      <c r="H88" s="104"/>
-      <c r="I88" s="104" t="s">
+      <c r="B93" s="113"/>
+      <c r="C93" s="113"/>
+      <c r="D93" s="113"/>
+      <c r="E93" s="113"/>
+      <c r="F93" s="113"/>
+      <c r="G93" s="113"/>
+      <c r="H93" s="113"/>
+      <c r="I93" s="113"/>
+      <c r="J93" s="113"/>
+      <c r="K93" s="113"/>
+      <c r="L93" s="114"/>
+    </row>
+    <row r="94" spans="1:12">
+      <c r="A94" s="115" t="s">
         <v>34</v>
       </c>
-      <c r="J88" s="104"/>
-      <c r="K88" s="104"/>
-      <c r="L88" s="107"/>
-    </row>
-    <row r="89" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A89" s="100"/>
-      <c r="B89" s="101"/>
-      <c r="C89" s="101"/>
-      <c r="D89" s="105"/>
-      <c r="E89" s="105"/>
-      <c r="F89" s="105"/>
-      <c r="G89" s="105"/>
-      <c r="H89" s="105"/>
-      <c r="I89" s="105"/>
-      <c r="J89" s="105"/>
-      <c r="K89" s="105"/>
-      <c r="L89" s="108"/>
-    </row>
-    <row r="90" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A90" s="100"/>
-      <c r="B90" s="101"/>
-      <c r="C90" s="101"/>
-      <c r="D90" s="105"/>
-      <c r="E90" s="105"/>
-      <c r="F90" s="105"/>
-      <c r="G90" s="105"/>
-      <c r="H90" s="105"/>
-      <c r="I90" s="105"/>
-      <c r="J90" s="105"/>
-      <c r="K90" s="105"/>
-      <c r="L90" s="108"/>
-    </row>
-    <row r="91" spans="1:12" ht="19.2" customHeight="1">
-      <c r="A91" s="102"/>
-      <c r="B91" s="103"/>
-      <c r="C91" s="103"/>
-      <c r="D91" s="106"/>
-      <c r="E91" s="106"/>
-      <c r="F91" s="106"/>
-      <c r="G91" s="106"/>
-      <c r="H91" s="106"/>
-      <c r="I91" s="106"/>
-      <c r="J91" s="106"/>
-      <c r="K91" s="106"/>
-      <c r="L91" s="109"/>
-    </row>
-    <row r="93" spans="1:12" ht="15.6">
-      <c r="A93" s="110" t="s">
+      <c r="B94" s="116"/>
+      <c r="C94" s="116"/>
+      <c r="D94" s="116"/>
+      <c r="E94" s="116"/>
+      <c r="F94" s="116"/>
+      <c r="G94" s="116"/>
+      <c r="H94" s="116"/>
+      <c r="I94" s="116"/>
+      <c r="J94" s="116"/>
+      <c r="K94" s="116"/>
+      <c r="L94" s="117"/>
+    </row>
+    <row r="95" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A95" s="127" t="s">
+        <v>39</v>
+      </c>
+      <c r="B95" s="128"/>
+      <c r="C95" s="128"/>
+      <c r="D95" s="128"/>
+      <c r="E95" s="128"/>
+      <c r="F95" s="128"/>
+      <c r="G95" s="128"/>
+      <c r="H95" s="128"/>
+      <c r="I95" s="128"/>
+      <c r="J95" s="128"/>
+      <c r="K95" s="128"/>
+      <c r="L95" s="129"/>
+    </row>
+    <row r="96" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A96" s="130"/>
+      <c r="B96" s="131"/>
+      <c r="C96" s="131"/>
+      <c r="D96" s="131"/>
+      <c r="E96" s="131"/>
+      <c r="F96" s="131"/>
+      <c r="G96" s="131"/>
+      <c r="H96" s="131"/>
+      <c r="I96" s="131"/>
+      <c r="J96" s="131"/>
+      <c r="K96" s="131"/>
+      <c r="L96" s="132"/>
+    </row>
+    <row r="97" spans="1:12" ht="13.8" customHeight="1">
+      <c r="A97" s="130"/>
+      <c r="B97" s="131"/>
+      <c r="C97" s="131"/>
+      <c r="D97" s="131"/>
+      <c r="E97" s="131"/>
+      <c r="F97" s="131"/>
+      <c r="G97" s="131"/>
+      <c r="H97" s="131"/>
+      <c r="I97" s="131"/>
+      <c r="J97" s="131"/>
+      <c r="K97" s="131"/>
+      <c r="L97" s="132"/>
+    </row>
+    <row r="98" spans="1:12" ht="13.2" hidden="1" customHeight="1">
+      <c r="A98" s="130"/>
+      <c r="B98" s="131"/>
+      <c r="C98" s="131"/>
+      <c r="D98" s="131"/>
+      <c r="E98" s="131"/>
+      <c r="F98" s="131"/>
+      <c r="G98" s="131"/>
+      <c r="H98" s="131"/>
+      <c r="I98" s="131"/>
+      <c r="J98" s="131"/>
+      <c r="K98" s="131"/>
+      <c r="L98" s="132"/>
+    </row>
+    <row r="99" spans="1:12" ht="18" hidden="1" customHeight="1">
+      <c r="A99" s="130"/>
+      <c r="B99" s="131"/>
+      <c r="C99" s="131"/>
+      <c r="D99" s="131"/>
+      <c r="E99" s="131"/>
+      <c r="F99" s="131"/>
+      <c r="G99" s="131"/>
+      <c r="H99" s="131"/>
+      <c r="I99" s="131"/>
+      <c r="J99" s="131"/>
+      <c r="K99" s="131"/>
+      <c r="L99" s="132"/>
+    </row>
+    <row r="100" spans="1:12" ht="18" hidden="1" customHeight="1">
+      <c r="A100" s="133"/>
+      <c r="B100" s="134"/>
+      <c r="C100" s="134"/>
+      <c r="D100" s="134"/>
+      <c r="E100" s="134"/>
+      <c r="F100" s="134"/>
+      <c r="G100" s="134"/>
+      <c r="H100" s="134"/>
+      <c r="I100" s="134"/>
+      <c r="J100" s="134"/>
+      <c r="K100" s="134"/>
+      <c r="L100" s="135"/>
+    </row>
+    <row r="102" spans="1:12">
+      <c r="A102" s="115" t="s">
         <v>35</v>
       </c>
-      <c r="B93" s="111"/>
-      <c r="C93" s="111"/>
-      <c r="D93" s="111"/>
-      <c r="E93" s="111"/>
-      <c r="F93" s="111"/>
-      <c r="G93" s="111"/>
-      <c r="H93" s="111"/>
-      <c r="I93" s="111"/>
-      <c r="J93" s="111"/>
-      <c r="K93" s="111"/>
-      <c r="L93" s="112"/>
-    </row>
-    <row r="94" spans="1:12">
-      <c r="A94" s="113" t="s">
+      <c r="B102" s="116"/>
+      <c r="C102" s="116"/>
+      <c r="D102" s="116"/>
+      <c r="E102" s="116"/>
+      <c r="F102" s="116"/>
+      <c r="G102" s="116"/>
+      <c r="H102" s="116"/>
+      <c r="I102" s="116"/>
+      <c r="J102" s="116"/>
+      <c r="K102" s="116"/>
+      <c r="L102" s="117"/>
+    </row>
+    <row r="103" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A103" s="127" t="s">
         <v>36</v>
       </c>
-      <c r="B94" s="114"/>
-      <c r="C94" s="114"/>
-      <c r="D94" s="114"/>
-      <c r="E94" s="114"/>
-      <c r="F94" s="114"/>
-      <c r="G94" s="114"/>
-      <c r="H94" s="114"/>
-      <c r="I94" s="114"/>
-      <c r="J94" s="114"/>
-      <c r="K94" s="114"/>
-      <c r="L94" s="115"/>
-    </row>
-    <row r="95" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A95" s="125" t="s">
-        <v>42</v>
-      </c>
-      <c r="B95" s="126"/>
-      <c r="C95" s="126"/>
-      <c r="D95" s="126"/>
-      <c r="E95" s="126"/>
-      <c r="F95" s="126"/>
-      <c r="G95" s="126"/>
-      <c r="H95" s="126"/>
-      <c r="I95" s="126"/>
-      <c r="J95" s="126"/>
-      <c r="K95" s="126"/>
-      <c r="L95" s="127"/>
-    </row>
-    <row r="96" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A96" s="128"/>
-      <c r="B96" s="129"/>
-      <c r="C96" s="129"/>
-      <c r="D96" s="129"/>
-      <c r="E96" s="129"/>
-      <c r="F96" s="129"/>
-      <c r="G96" s="129"/>
-      <c r="H96" s="129"/>
-      <c r="I96" s="129"/>
-      <c r="J96" s="129"/>
-      <c r="K96" s="129"/>
-      <c r="L96" s="130"/>
-    </row>
-    <row r="97" spans="1:12" ht="13.8" customHeight="1">
-      <c r="A97" s="128"/>
-      <c r="B97" s="129"/>
-      <c r="C97" s="129"/>
-      <c r="D97" s="129"/>
-      <c r="E97" s="129"/>
-      <c r="F97" s="129"/>
-      <c r="G97" s="129"/>
-      <c r="H97" s="129"/>
-      <c r="I97" s="129"/>
-      <c r="J97" s="129"/>
-      <c r="K97" s="129"/>
-      <c r="L97" s="130"/>
-    </row>
-    <row r="98" spans="1:12" ht="13.2" hidden="1" customHeight="1">
-      <c r="A98" s="128"/>
-      <c r="B98" s="129"/>
-      <c r="C98" s="129"/>
-      <c r="D98" s="129"/>
-      <c r="E98" s="129"/>
-      <c r="F98" s="129"/>
-      <c r="G98" s="129"/>
-      <c r="H98" s="129"/>
-      <c r="I98" s="129"/>
-      <c r="J98" s="129"/>
-      <c r="K98" s="129"/>
-      <c r="L98" s="130"/>
-    </row>
-    <row r="99" spans="1:12" ht="18" hidden="1" customHeight="1">
-      <c r="A99" s="128"/>
-      <c r="B99" s="129"/>
-      <c r="C99" s="129"/>
-      <c r="D99" s="129"/>
-      <c r="E99" s="129"/>
-      <c r="F99" s="129"/>
-      <c r="G99" s="129"/>
-      <c r="H99" s="129"/>
-      <c r="I99" s="129"/>
-      <c r="J99" s="129"/>
-      <c r="K99" s="129"/>
-      <c r="L99" s="130"/>
-    </row>
-    <row r="100" spans="1:12" ht="18" hidden="1" customHeight="1">
-      <c r="A100" s="131"/>
-      <c r="B100" s="132"/>
-      <c r="C100" s="132"/>
-      <c r="D100" s="132"/>
-      <c r="E100" s="132"/>
-      <c r="F100" s="132"/>
-      <c r="G100" s="132"/>
-      <c r="H100" s="132"/>
-      <c r="I100" s="132"/>
-      <c r="J100" s="132"/>
-      <c r="K100" s="132"/>
-      <c r="L100" s="133"/>
-    </row>
-    <row r="102" spans="1:12">
-      <c r="A102" s="113" t="s">
+      <c r="B103" s="128"/>
+      <c r="C103" s="128"/>
+      <c r="D103" s="128"/>
+      <c r="E103" s="128"/>
+      <c r="F103" s="128"/>
+      <c r="G103" s="128"/>
+      <c r="H103" s="128"/>
+      <c r="I103" s="128"/>
+      <c r="J103" s="128"/>
+      <c r="K103" s="128"/>
+      <c r="L103" s="129"/>
+    </row>
+    <row r="104" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A104" s="130"/>
+      <c r="B104" s="131"/>
+      <c r="C104" s="131"/>
+      <c r="D104" s="131"/>
+      <c r="E104" s="131"/>
+      <c r="F104" s="131"/>
+      <c r="G104" s="131"/>
+      <c r="H104" s="131"/>
+      <c r="I104" s="131"/>
+      <c r="J104" s="131"/>
+      <c r="K104" s="131"/>
+      <c r="L104" s="132"/>
+    </row>
+    <row r="105" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A105" s="130"/>
+      <c r="B105" s="131"/>
+      <c r="C105" s="131"/>
+      <c r="D105" s="131"/>
+      <c r="E105" s="131"/>
+      <c r="F105" s="131"/>
+      <c r="G105" s="131"/>
+      <c r="H105" s="131"/>
+      <c r="I105" s="131"/>
+      <c r="J105" s="131"/>
+      <c r="K105" s="131"/>
+      <c r="L105" s="132"/>
+    </row>
+    <row r="106" spans="1:12" ht="18" hidden="1" customHeight="1">
+      <c r="A106" s="130"/>
+      <c r="B106" s="131"/>
+      <c r="C106" s="131"/>
+      <c r="D106" s="131"/>
+      <c r="E106" s="131"/>
+      <c r="F106" s="131"/>
+      <c r="G106" s="131"/>
+      <c r="H106" s="131"/>
+      <c r="I106" s="131"/>
+      <c r="J106" s="131"/>
+      <c r="K106" s="131"/>
+      <c r="L106" s="132"/>
+    </row>
+    <row r="107" spans="1:12" ht="18" hidden="1" customHeight="1">
+      <c r="A107" s="130"/>
+      <c r="B107" s="131"/>
+      <c r="C107" s="131"/>
+      <c r="D107" s="131"/>
+      <c r="E107" s="131"/>
+      <c r="F107" s="131"/>
+      <c r="G107" s="131"/>
+      <c r="H107" s="131"/>
+      <c r="I107" s="131"/>
+      <c r="J107" s="131"/>
+      <c r="K107" s="131"/>
+      <c r="L107" s="132"/>
+    </row>
+    <row r="108" spans="1:12" ht="18" hidden="1" customHeight="1">
+      <c r="A108" s="133"/>
+      <c r="B108" s="134"/>
+      <c r="C108" s="134"/>
+      <c r="D108" s="134"/>
+      <c r="E108" s="134"/>
+      <c r="F108" s="134"/>
+      <c r="G108" s="134"/>
+      <c r="H108" s="134"/>
+      <c r="I108" s="134"/>
+      <c r="J108" s="134"/>
+      <c r="K108" s="134"/>
+      <c r="L108" s="135"/>
+    </row>
+    <row r="110" spans="1:12">
+      <c r="A110" s="115" t="s">
         <v>37</v>
       </c>
-      <c r="B102" s="114"/>
-      <c r="C102" s="114"/>
-      <c r="D102" s="114"/>
-      <c r="E102" s="114"/>
-      <c r="F102" s="114"/>
-      <c r="G102" s="114"/>
-      <c r="H102" s="114"/>
-      <c r="I102" s="114"/>
-      <c r="J102" s="114"/>
-      <c r="K102" s="114"/>
-      <c r="L102" s="115"/>
-    </row>
-    <row r="103" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A103" s="125" t="s">
+      <c r="B110" s="116"/>
+      <c r="C110" s="116"/>
+      <c r="D110" s="116"/>
+      <c r="E110" s="116"/>
+      <c r="F110" s="116"/>
+      <c r="G110" s="116"/>
+      <c r="H110" s="116"/>
+      <c r="I110" s="116"/>
+      <c r="J110" s="116"/>
+      <c r="K110" s="116"/>
+      <c r="L110" s="117"/>
+    </row>
+    <row r="111" spans="1:12" ht="18.45" customHeight="1">
+      <c r="A111" s="127" t="s">
         <v>38</v>
       </c>
-      <c r="B103" s="126"/>
-      <c r="C103" s="126"/>
-      <c r="D103" s="126"/>
-      <c r="E103" s="126"/>
-      <c r="F103" s="126"/>
-      <c r="G103" s="126"/>
-      <c r="H103" s="126"/>
-      <c r="I103" s="126"/>
-      <c r="J103" s="126"/>
-      <c r="K103" s="126"/>
-      <c r="L103" s="127"/>
-    </row>
-    <row r="104" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A104" s="128"/>
-      <c r="B104" s="129"/>
-      <c r="C104" s="129"/>
-      <c r="D104" s="129"/>
-      <c r="E104" s="129"/>
-      <c r="F104" s="129"/>
-      <c r="G104" s="129"/>
-      <c r="H104" s="129"/>
-      <c r="I104" s="129"/>
-      <c r="J104" s="129"/>
-      <c r="K104" s="129"/>
-      <c r="L104" s="130"/>
-    </row>
-    <row r="105" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A105" s="128"/>
-      <c r="B105" s="129"/>
-      <c r="C105" s="129"/>
-      <c r="D105" s="129"/>
-      <c r="E105" s="129"/>
-      <c r="F105" s="129"/>
-      <c r="G105" s="129"/>
-      <c r="H105" s="129"/>
-      <c r="I105" s="129"/>
-      <c r="J105" s="129"/>
-      <c r="K105" s="129"/>
-      <c r="L105" s="130"/>
-    </row>
-    <row r="106" spans="1:12" ht="18" hidden="1" customHeight="1">
-      <c r="A106" s="128"/>
-      <c r="B106" s="129"/>
-      <c r="C106" s="129"/>
-      <c r="D106" s="129"/>
-      <c r="E106" s="129"/>
-      <c r="F106" s="129"/>
-      <c r="G106" s="129"/>
-      <c r="H106" s="129"/>
-      <c r="I106" s="129"/>
-      <c r="J106" s="129"/>
-      <c r="K106" s="129"/>
-      <c r="L106" s="130"/>
-    </row>
-    <row r="107" spans="1:12" ht="18" hidden="1" customHeight="1">
-      <c r="A107" s="128"/>
-      <c r="B107" s="129"/>
-      <c r="C107" s="129"/>
-      <c r="D107" s="129"/>
-      <c r="E107" s="129"/>
-      <c r="F107" s="129"/>
-      <c r="G107" s="129"/>
-      <c r="H107" s="129"/>
-      <c r="I107" s="129"/>
-      <c r="J107" s="129"/>
-      <c r="K107" s="129"/>
-      <c r="L107" s="130"/>
-    </row>
-    <row r="108" spans="1:12" ht="18" hidden="1" customHeight="1">
-      <c r="A108" s="131"/>
-      <c r="B108" s="132"/>
-      <c r="C108" s="132"/>
-      <c r="D108" s="132"/>
-      <c r="E108" s="132"/>
-      <c r="F108" s="132"/>
-      <c r="G108" s="132"/>
-      <c r="H108" s="132"/>
-      <c r="I108" s="132"/>
-      <c r="J108" s="132"/>
-      <c r="K108" s="132"/>
-      <c r="L108" s="133"/>
-    </row>
-    <row r="110" spans="1:12">
-      <c r="A110" s="113" t="s">
-        <v>39</v>
-      </c>
-      <c r="B110" s="114"/>
-      <c r="C110" s="114"/>
-      <c r="D110" s="114"/>
-      <c r="E110" s="114"/>
-      <c r="F110" s="114"/>
-      <c r="G110" s="114"/>
-      <c r="H110" s="114"/>
-      <c r="I110" s="114"/>
-      <c r="J110" s="114"/>
-      <c r="K110" s="114"/>
-      <c r="L110" s="115"/>
-    </row>
-    <row r="111" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A111" s="125" t="s">
-        <v>40</v>
-      </c>
-      <c r="B111" s="126"/>
-      <c r="C111" s="126"/>
-      <c r="D111" s="126"/>
-      <c r="E111" s="126"/>
-      <c r="F111" s="126"/>
-      <c r="G111" s="126"/>
-      <c r="H111" s="126"/>
-      <c r="I111" s="126"/>
-      <c r="J111" s="126"/>
-      <c r="K111" s="126"/>
-      <c r="L111" s="127"/>
+      <c r="B111" s="128"/>
+      <c r="C111" s="128"/>
+      <c r="D111" s="128"/>
+      <c r="E111" s="128"/>
+      <c r="F111" s="128"/>
+      <c r="G111" s="128"/>
+      <c r="H111" s="128"/>
+      <c r="I111" s="128"/>
+      <c r="J111" s="128"/>
+      <c r="K111" s="128"/>
+      <c r="L111" s="129"/>
     </row>
     <row r="112" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A112" s="128"/>
-      <c r="B112" s="129"/>
-      <c r="C112" s="129"/>
-      <c r="D112" s="129"/>
-      <c r="E112" s="129"/>
-      <c r="F112" s="129"/>
-      <c r="G112" s="129"/>
-      <c r="H112" s="129"/>
-      <c r="I112" s="129"/>
-      <c r="J112" s="129"/>
-      <c r="K112" s="129"/>
-      <c r="L112" s="130"/>
+      <c r="A112" s="130"/>
+      <c r="B112" s="131"/>
+      <c r="C112" s="131"/>
+      <c r="D112" s="131"/>
+      <c r="E112" s="131"/>
+      <c r="F112" s="131"/>
+      <c r="G112" s="131"/>
+      <c r="H112" s="131"/>
+      <c r="I112" s="131"/>
+      <c r="J112" s="131"/>
+      <c r="K112" s="131"/>
+      <c r="L112" s="132"/>
     </row>
     <row r="113" spans="1:12" ht="18.45" customHeight="1">
-      <c r="A113" s="128"/>
-      <c r="B113" s="129"/>
-      <c r="C113" s="129"/>
-      <c r="D113" s="129"/>
-      <c r="E113" s="129"/>
-      <c r="F113" s="129"/>
-      <c r="G113" s="129"/>
-      <c r="H113" s="129"/>
-      <c r="I113" s="129"/>
-      <c r="J113" s="129"/>
-      <c r="K113" s="129"/>
-      <c r="L113" s="130"/>
+      <c r="A113" s="130"/>
+      <c r="B113" s="131"/>
+      <c r="C113" s="131"/>
+      <c r="D113" s="131"/>
+      <c r="E113" s="131"/>
+      <c r="F113" s="131"/>
+      <c r="G113" s="131"/>
+      <c r="H113" s="131"/>
+      <c r="I113" s="131"/>
+      <c r="J113" s="131"/>
+      <c r="K113" s="131"/>
+      <c r="L113" s="132"/>
     </row>
     <row r="114" spans="1:12" ht="1.2" customHeight="1">
-      <c r="A114" s="128"/>
-      <c r="B114" s="129"/>
-      <c r="C114" s="129"/>
-      <c r="D114" s="129"/>
-      <c r="E114" s="129"/>
-      <c r="F114" s="129"/>
-      <c r="G114" s="129"/>
-      <c r="H114" s="129"/>
-      <c r="I114" s="129"/>
-      <c r="J114" s="129"/>
-      <c r="K114" s="129"/>
-      <c r="L114" s="130"/>
+      <c r="A114" s="130"/>
+      <c r="B114" s="131"/>
+      <c r="C114" s="131"/>
+      <c r="D114" s="131"/>
+      <c r="E114" s="131"/>
+      <c r="F114" s="131"/>
+      <c r="G114" s="131"/>
+      <c r="H114" s="131"/>
+      <c r="I114" s="131"/>
+      <c r="J114" s="131"/>
+      <c r="K114" s="131"/>
+      <c r="L114" s="132"/>
     </row>
     <row r="115" spans="1:12" ht="18" hidden="1" customHeight="1">
-      <c r="A115" s="128"/>
-      <c r="B115" s="129"/>
-      <c r="C115" s="129"/>
-      <c r="D115" s="129"/>
-      <c r="E115" s="129"/>
-      <c r="F115" s="129"/>
-      <c r="G115" s="129"/>
-      <c r="H115" s="129"/>
-      <c r="I115" s="129"/>
-      <c r="J115" s="129"/>
-      <c r="K115" s="129"/>
-      <c r="L115" s="130"/>
+      <c r="A115" s="130"/>
+      <c r="B115" s="131"/>
+      <c r="C115" s="131"/>
+      <c r="D115" s="131"/>
+      <c r="E115" s="131"/>
+      <c r="F115" s="131"/>
+      <c r="G115" s="131"/>
+      <c r="H115" s="131"/>
+      <c r="I115" s="131"/>
+      <c r="J115" s="131"/>
+      <c r="K115" s="131"/>
+      <c r="L115" s="132"/>
     </row>
     <row r="116" spans="1:12" ht="18" hidden="1" customHeight="1">
-      <c r="A116" s="131"/>
-      <c r="B116" s="132"/>
-      <c r="C116" s="132"/>
-      <c r="D116" s="132"/>
-      <c r="E116" s="132"/>
-      <c r="F116" s="132"/>
-      <c r="G116" s="132"/>
-      <c r="H116" s="132"/>
-      <c r="I116" s="132"/>
-      <c r="J116" s="132"/>
-      <c r="K116" s="132"/>
-      <c r="L116" s="133"/>
+      <c r="A116" s="133"/>
+      <c r="B116" s="134"/>
+      <c r="C116" s="134"/>
+      <c r="D116" s="134"/>
+      <c r="E116" s="134"/>
+      <c r="F116" s="134"/>
+      <c r="G116" s="134"/>
+      <c r="H116" s="134"/>
+      <c r="I116" s="134"/>
+      <c r="J116" s="134"/>
+      <c r="K116" s="134"/>
+      <c r="L116" s="135"/>
     </row>
     <row r="118" spans="1:12" s="1" customFormat="1" ht="0.6" customHeight="1">
-      <c r="A118" s="116"/>
-      <c r="B118" s="117"/>
-      <c r="C118" s="117"/>
-      <c r="D118" s="117"/>
-      <c r="E118" s="117"/>
-      <c r="F118" s="117"/>
-      <c r="G118" s="117"/>
-      <c r="H118" s="117"/>
-      <c r="I118" s="117"/>
-      <c r="J118" s="117"/>
-      <c r="K118" s="117"/>
-      <c r="L118" s="118"/>
+      <c r="A118" s="118"/>
+      <c r="B118" s="119"/>
+      <c r="C118" s="119"/>
+      <c r="D118" s="119"/>
+      <c r="E118" s="119"/>
+      <c r="F118" s="119"/>
+      <c r="G118" s="119"/>
+      <c r="H118" s="119"/>
+      <c r="I118" s="119"/>
+      <c r="J118" s="119"/>
+      <c r="K118" s="119"/>
+      <c r="L118" s="120"/>
     </row>
     <row r="119" spans="1:12" ht="2.4" hidden="1" customHeight="1">
-      <c r="A119" s="119"/>
-      <c r="B119" s="120"/>
-      <c r="C119" s="120"/>
-      <c r="D119" s="120"/>
-      <c r="E119" s="120"/>
-      <c r="F119" s="120"/>
-      <c r="G119" s="120"/>
-      <c r="H119" s="120"/>
-      <c r="I119" s="120"/>
-      <c r="J119" s="120"/>
-      <c r="K119" s="120"/>
-      <c r="L119" s="121"/>
+      <c r="A119" s="121"/>
+      <c r="B119" s="122"/>
+      <c r="C119" s="122"/>
+      <c r="D119" s="122"/>
+      <c r="E119" s="122"/>
+      <c r="F119" s="122"/>
+      <c r="G119" s="122"/>
+      <c r="H119" s="122"/>
+      <c r="I119" s="122"/>
+      <c r="J119" s="122"/>
+      <c r="K119" s="122"/>
+      <c r="L119" s="123"/>
     </row>
     <row r="120" spans="1:12" s="1" customFormat="1" hidden="1">
-      <c r="A120" s="122"/>
-      <c r="B120" s="123"/>
-      <c r="C120" s="123"/>
-      <c r="D120" s="123"/>
-      <c r="E120" s="123"/>
-      <c r="F120" s="123"/>
-      <c r="G120" s="123"/>
-      <c r="H120" s="123"/>
-      <c r="I120" s="123"/>
-      <c r="J120" s="123"/>
-      <c r="K120" s="123"/>
-      <c r="L120" s="124"/>
+      <c r="A120" s="124"/>
+      <c r="B120" s="125"/>
+      <c r="C120" s="125"/>
+      <c r="D120" s="125"/>
+      <c r="E120" s="125"/>
+      <c r="F120" s="125"/>
+      <c r="G120" s="125"/>
+      <c r="H120" s="125"/>
+      <c r="I120" s="125"/>
+      <c r="J120" s="125"/>
+      <c r="K120" s="125"/>
+      <c r="L120" s="126"/>
     </row>
   </sheetData>
   <mergeCells count="49">

</xml_diff>